<commit_message>
Atualização automática convênios de entrada
</commit_message>
<xml_diff>
--- a/link_convenios.xlsx
+++ b/link_convenios.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\CGE\bi_atualizacao\portal_convenios_entrada\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m11483500\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2533" uniqueCount="1150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2541" uniqueCount="1154">
   <si>
     <t>https://drive.google.com/file/d/1mnH14gEK5_xghzIJ-rHHZ8lOxqCsVnB8/view</t>
   </si>
@@ -3491,6 +3491,18 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/1MPDAU1yAEIyTEt7-SFKo2NejDhqNUj2O/view</t>
+  </si>
+  <si>
+    <t>https://nuvem.cge.mg.gov.br/index.php/s/3je8MbXPHTMPiH2</t>
+  </si>
+  <si>
+    <t>https://nuvem.cge.mg.gov.br/index.php/s/ezRekmfGzw7TqS4</t>
+  </si>
+  <si>
+    <t>https://nuvem.cge.mg.gov.br/index.php/s/FdP7CXTxzcXJnn4</t>
+  </si>
+  <si>
+    <t>https://nuvem.cge.mg.gov.br/index.php/s/wyiceeaoCd2nQbD</t>
   </si>
 </sst>
 </file>
@@ -14322,6 +14334,12 @@
       <c r="A1023">
         <v>9461431</v>
       </c>
+      <c r="B1023" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C1023" t="s">
+        <v>891</v>
+      </c>
     </row>
     <row r="1024" spans="1:3">
       <c r="A1024">
@@ -14338,15 +14356,33 @@
       <c r="A1025">
         <v>9461433</v>
       </c>
+      <c r="B1025" t="s">
+        <v>1151</v>
+      </c>
+      <c r="C1025" t="s">
+        <v>891</v>
+      </c>
     </row>
     <row r="1026" spans="1:3">
       <c r="A1026">
         <v>9461434</v>
       </c>
+      <c r="B1026" t="s">
+        <v>1153</v>
+      </c>
+      <c r="C1026" t="s">
+        <v>891</v>
+      </c>
     </row>
     <row r="1027" spans="1:3">
       <c r="A1027">
         <v>9461435</v>
+      </c>
+      <c r="B1027" t="s">
+        <v>1150</v>
+      </c>
+      <c r="C1027" t="s">
+        <v>891</v>
       </c>
     </row>
     <row r="1028" spans="1:3">

</xml_diff>